<commit_message>
Honors and Services added
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitendra/Git Projects/jitendrakv.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815F81FC-3370-854A-857D-7D71AB7C11B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80A82BF7-3E94-5D4A-9E1D-94FD321E570E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="19060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="19060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PhD" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="203">
   <si>
     <t>Category</t>
   </si>
@@ -614,6 +614,24 @@
   </si>
   <si>
     <t>Nokia, USA</t>
+  </si>
+  <si>
+    <t>RohitPhD.jpg</t>
+  </si>
+  <si>
+    <t>AmitMTech2026.jpg</t>
+  </si>
+  <si>
+    <t>StutiMTech2027.jpg</t>
+  </si>
+  <si>
+    <t>hanna.jpg</t>
+  </si>
+  <si>
+    <t>IILM University Greater Noida, India</t>
+  </si>
+  <si>
+    <t>Samsung</t>
   </si>
 </sst>
 </file>
@@ -1086,6 +1104,9 @@
       <c r="D6" t="s">
         <v>12</v>
       </c>
+      <c r="I6" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1186,6 +1207,9 @@
       <c r="E2" t="s">
         <v>12</v>
       </c>
+      <c r="H2" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1288,6 +1312,12 @@
       <c r="E8" t="s">
         <v>42</v>
       </c>
+      <c r="F8" t="s">
+        <v>201</v>
+      </c>
+      <c r="H8" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1304,6 +1334,9 @@
       </c>
       <c r="E9" t="s">
         <v>42</v>
+      </c>
+      <c r="F9" t="s">
+        <v>202</v>
       </c>
       <c r="J9" t="s">
         <v>45</v>
@@ -2586,6 +2619,9 @@
       <c r="G6" t="s">
         <v>181</v>
       </c>
+      <c r="I6" t="s">
+        <v>200</v>
+      </c>
       <c r="K6" t="s">
         <v>182</v>
       </c>

</xml_diff>

<commit_message>
Student card formatting fix
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git Projects\jitendrakv.github.io\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitendra/Git Projects/jitendrakv.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05A28F07-2E76-4AAD-9375-81F1AB895BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B2ABCDB-EF54-0442-918F-AC91FE18B029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PhD" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="211">
   <si>
     <t>Name</t>
   </si>
@@ -656,6 +656,9 @@
   </si>
   <si>
     <t>NIT Tiruchirappalli, India</t>
+  </si>
+  <si>
+    <t>Synchrony Financial Services</t>
   </si>
 </sst>
 </file>
@@ -1035,22 +1038,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="18.6640625" customWidth="1"/>
     <col min="9" max="9" width="34" customWidth="1"/>
-    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1088,7 +1091,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1103,7 +1106,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1118,7 +1121,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1133,7 +1136,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1148,7 +1151,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1166,7 +1169,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1181,7 +1184,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1218,22 +1221,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD4758E0-2E06-CD49-AFCA-FFAEED49AC86}">
   <dimension ref="A1:K63"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="5"/>
-    <col min="5" max="5" width="111.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="5"/>
+    <col min="5" max="5" width="111.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" customWidth="1"/>
     <col min="10" max="10" width="0" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1268,7 +1271,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1291,7 +1294,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1311,7 +1314,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1331,7 +1334,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1371,7 +1374,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1391,7 +1394,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -1417,7 +1420,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -1443,7 +1446,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -1466,7 +1469,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -1512,7 +1515,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -1535,7 +1538,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>54</v>
       </c>
@@ -1558,7 +1561,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1581,7 +1584,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>56</v>
       </c>
@@ -1604,7 +1607,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>58</v>
       </c>
@@ -1627,7 +1630,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -1650,7 +1653,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -1673,7 +1676,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -1699,7 +1702,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -1722,7 +1725,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -1748,7 +1751,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -1771,7 +1774,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1794,7 +1797,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>73</v>
       </c>
@@ -1837,7 +1840,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1860,7 +1863,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>78</v>
       </c>
@@ -1883,7 +1886,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -1906,7 +1909,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>82</v>
       </c>
@@ -1929,7 +1932,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>87</v>
       </c>
@@ -1952,7 +1955,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>89</v>
       </c>
@@ -1975,7 +1978,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>91</v>
       </c>
@@ -1998,7 +2001,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>93</v>
       </c>
@@ -2021,7 +2024,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>95</v>
       </c>
@@ -2044,7 +2047,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>97</v>
       </c>
@@ -2073,7 +2076,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>99</v>
       </c>
@@ -2096,7 +2099,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>101</v>
       </c>
@@ -2119,7 +2122,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>103</v>
       </c>
@@ -2142,7 +2145,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>105</v>
       </c>
@@ -2165,7 +2168,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>107</v>
       </c>
@@ -2188,7 +2191,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>111</v>
       </c>
@@ -2208,7 +2211,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>113</v>
       </c>
@@ -2231,7 +2234,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>115</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>117</v>
       </c>
@@ -2274,7 +2277,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>119</v>
       </c>
@@ -2294,7 +2297,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>121</v>
       </c>
@@ -2314,7 +2317,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>123</v>
       </c>
@@ -2334,7 +2337,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>125</v>
       </c>
@@ -2354,7 +2357,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>127</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>129</v>
       </c>
@@ -2397,7 +2400,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>131</v>
       </c>
@@ -2417,7 +2420,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>133</v>
       </c>
@@ -2440,7 +2443,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>135</v>
       </c>
@@ -2460,7 +2463,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>138</v>
       </c>
@@ -2479,8 +2482,11 @@
       <c r="F55" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G55" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>139</v>
       </c>
@@ -2503,7 +2509,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>140</v>
       </c>
@@ -2523,7 +2529,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>142</v>
       </c>
@@ -2543,7 +2549,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -2566,7 +2572,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>147</v>
       </c>
@@ -2589,7 +2595,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>149</v>
       </c>
@@ -2612,7 +2618,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>151</v>
       </c>
@@ -2635,7 +2641,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>153</v>
       </c>
@@ -2668,9 +2674,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA0CB0B7-D58C-1941-ACD1-F59BFD833B36}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2705,7 +2711,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>156</v>
       </c>
@@ -2725,7 +2731,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>159</v>
       </c>
@@ -2753,13 +2759,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6960067F-0CCA-7C4D-BA1D-1D24D0A75DDF}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="7" width="45" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="66.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="66.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2794,7 +2800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>162</v>
       </c>
@@ -2817,7 +2823,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>164</v>
       </c>
@@ -2840,7 +2846,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>165</v>
       </c>
@@ -2863,7 +2869,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>168</v>
       </c>
@@ -2886,7 +2892,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>171</v>
       </c>

</xml_diff>